<commit_message>
load classification datasets from file
</commit_message>
<xml_diff>
--- a/resources/HENRY_OPERA.xlsx
+++ b/resources/HENRY_OPERA.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8616"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8616" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Training" sheetId="3" r:id="rId1"/>
@@ -11692,12 +11692,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -11727,11 +11733,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12036,6 +12043,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P592"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -24788,52 +24798,52 @@
       </c>
     </row>
     <row r="256" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A256">
+      <c r="A256" s="2">
         <v>256</v>
       </c>
-      <c r="B256" t="s">
+      <c r="B256" s="2" t="s">
         <v>1833</v>
       </c>
-      <c r="C256" t="s">
+      <c r="C256" s="2" t="s">
         <v>1834</v>
       </c>
-      <c r="D256" t="s">
+      <c r="D256" s="2" t="s">
         <v>1835</v>
       </c>
-      <c r="E256" t="s">
+      <c r="E256" s="2" t="s">
         <v>1836</v>
       </c>
-      <c r="F256" t="s">
+      <c r="F256" s="2" t="s">
         <v>1837</v>
       </c>
-      <c r="G256" t="s">
-        <v>28</v>
-      </c>
-      <c r="H256" t="s">
-        <v>28</v>
-      </c>
-      <c r="I256" t="s">
+      <c r="G256" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H256" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I256" s="2" t="s">
         <v>1838</v>
       </c>
-      <c r="J256" t="s">
+      <c r="J256" s="2" t="s">
         <v>1685</v>
       </c>
-      <c r="K256" t="s">
+      <c r="K256" s="2" t="s">
         <v>1838</v>
       </c>
-      <c r="L256" t="s">
-        <v>28</v>
-      </c>
-      <c r="M256" t="s">
-        <v>37</v>
-      </c>
-      <c r="N256" t="s">
-        <v>38</v>
-      </c>
-      <c r="O256" t="s">
+      <c r="L256" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M256" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N256" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O256" s="2" t="s">
         <v>1839</v>
       </c>
-      <c r="P256">
+      <c r="P256" s="2">
         <v>-2.1719849357760199</v>
       </c>
     </row>
@@ -26237,53 +26247,53 @@
         <v>-5.0716041477433</v>
       </c>
     </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A285">
+    <row r="285" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A285" s="2">
         <v>285</v>
       </c>
-      <c r="B285" t="s">
+      <c r="B285" s="2" t="s">
         <v>2026</v>
       </c>
-      <c r="C285" t="s">
+      <c r="C285" s="2" t="s">
         <v>1834</v>
       </c>
-      <c r="D285" t="s">
+      <c r="D285" s="2" t="s">
         <v>1835</v>
       </c>
-      <c r="E285" t="s">
+      <c r="E285" s="2" t="s">
         <v>1836</v>
       </c>
-      <c r="F285" t="s">
+      <c r="F285" s="2" t="s">
         <v>1837</v>
       </c>
-      <c r="G285" t="s">
-        <v>28</v>
-      </c>
-      <c r="H285" t="s">
-        <v>28</v>
-      </c>
-      <c r="I285" t="s">
+      <c r="G285" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H285" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I285" s="2" t="s">
         <v>1838</v>
       </c>
-      <c r="J285" t="s">
+      <c r="J285" s="2" t="s">
         <v>1685</v>
       </c>
-      <c r="K285" t="s">
+      <c r="K285" s="2" t="s">
         <v>1838</v>
       </c>
-      <c r="L285" t="s">
-        <v>28</v>
-      </c>
-      <c r="M285" t="s">
-        <v>37</v>
-      </c>
-      <c r="N285" t="s">
-        <v>38</v>
-      </c>
-      <c r="O285" t="s">
+      <c r="L285" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M285" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N285" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O285" s="2" t="s">
         <v>2027</v>
       </c>
-      <c r="P285">
+      <c r="P285" s="2">
         <v>-2.38933983691012</v>
       </c>
     </row>

</xml_diff>